<commit_message>
feat: add turnover_time field and template column
Operation.turnover_time defaults to 0.0 so every existing construction
site keeps its current behavior. The operations sheet gains
turnover_time_hrs directly after processing_time_hrs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/instance_template.xlsx
+++ b/docs/instance_template.xlsx
@@ -11,13 +11,14 @@
     <sheet name="orders" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="tasks" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="operations" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="machine_types" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="machines" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="tooling_types" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="toolings" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="personnel" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="downtimes" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="instructions" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="initial_state" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="machine_types" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="machines" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="tooling_types" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="toolings" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="personnel" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="downtimes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="instructions" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026.03.26</t>
+          <t>2026.07.16.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -470,7 +471,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>所有相对时间默认都以 plan_start_at 为锚点；也支持直接填写 ISO 8601 日期时间。</t>
+          <t>All time fields may be hour offsets from plan_start_at, or ISO 8601 datetimes.</t>
         </is>
       </c>
     </row>
@@ -480,6 +481,114 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>personnel_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>personnel_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>shifts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PS-turning-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Turning-operator-1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>skill_turning</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0/8/10;0/20/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PS-milling-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Milling-operator-1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>skill_milling</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0/8/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PS-assembly-01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Assembly-operator-1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>skill_assembly</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0/8/10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -557,13 +666,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -578,7 +687,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>说明</t>
+          <t>description</t>
         </is>
       </c>
     </row>
@@ -590,7 +699,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>当前模板版本为 2026.03.26。</t>
+          <t>Current template version: 2026.07.16.1</t>
         </is>
       </c>
     </row>
@@ -602,7 +711,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>orders/tasks/downtimes 的时间既可以填写相对 plan_start_at 的小时数，也可以直接填写 ISO 8601 日期时间。</t>
+          <t>Orders, tasks, downtimes and initial_state time fields can be hour offsets from plan_start_at, or ISO 8601 datetimes.</t>
         </is>
       </c>
     </row>
@@ -614,7 +723,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>任务层 due_date 可留空，导入时会自动继承所属订单 due_date。</t>
+          <t>Task due_date may be blank and will inherit the parent order due_date during import.</t>
         </is>
       </c>
     </row>
@@ -626,7 +735,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>任务层 release_time 可留空，导入时会自动继承所属订单 release_time。</t>
+          <t>Task release_time may be blank and will inherit the parent order release_time during import.</t>
         </is>
       </c>
     </row>
@@ -638,67 +747,103 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>导入或生成实例后，系统会基于订单交期、任务/BOM 依赖和工序前后关系，自动反推任务与工序的理想最晚开始/完成时间，无需人工填写。</t>
+          <t>After generation or import, the system derives internal latest start/finish targets from order due dates, BOM/task dependencies and operation precedence.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>shifts</t>
+          <t>initial_state</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>班次格式为 day/start_hour/hours；多个班次用分号分隔，例如 0/8/10;0/20/8。</t>
+          <t>Use the initial_state sheet to describe the shop-floor state at the planning anchor: pending, ready, processing or completed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>processing state</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>人员 skills 支持多个技能，使用分号分隔，例如 skill_turning;skill_milling。</t>
+          <t>For processing rows, fill at least initial_assigned_machine_id. You may provide remaining productive hours, or provide initial_end_time to express that the resources are occupied until that time.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>eligible_machine_ids</t>
+          <t>completed state</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>多个设备 ID 使用分号分隔；留空时按 process_type 匹配 machine_types。</t>
+          <t>Completed operations are treated as already done before the simulation/optimization starts, so downstream work can start immediately when other dependencies are satisfied.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>required resources</t>
+          <t>shifts</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>required_tooling_types 与 required_personnel_skills 均支持多值分号分隔。</t>
+          <t>Shift format is day/start_hour/hours; multiple shifts are separated by semicolons, for example 0/8/10;0/20/8.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Personnel skills support multiple values separated by semicolons, for example skill_turning;skill_milling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>eligible_machine_ids</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Multiple machine IDs are separated by semicolons; if blank, machines are matched by process_type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>required resources</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>required_tooling_types and required_personnel_skills both support multiple semicolon-separated values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>resource sheets</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>tooling_types、toolings、personnel、downtimes 四个 sheet 是当前版本的关键资源配置页。</t>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tooling_types, toolings, personnel, downtimes and initial_state are the key resource/state sheets in this template.</t>
         </is>
       </c>
     </row>
@@ -758,7 +903,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>订单-1</t>
+          <t>Order-1</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -779,7 +924,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>订单-2</t>
+          <t>Order-2</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -808,7 +953,7 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -865,7 +1010,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>子件-1</t>
+          <t>Part-1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -890,7 +1035,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>装配主任务</t>
+          <t>Assembly-main</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -917,7 +1062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -925,11 +1070,12 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -960,25 +1106,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>turnover_time_hrs</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>predecessor_ops</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>predecessor_tasks</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>eligible_machine_ids</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>required_tooling_types</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>required_personnel_skills</t>
         </is>
@@ -997,7 +1148,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>车削工序</t>
+          <t>Turning</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1008,19 +1159,22 @@
       <c r="E2" t="n">
         <v>5.5</v>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
         <is>
           <t>turning_1;turning_2</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>tool_turning</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>skill_turning</t>
         </is>
@@ -1039,7 +1193,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>铣削工序</t>
+          <t>Milling</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1050,23 +1204,26 @@
       <c r="E3" t="n">
         <v>3.2</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>OP-0001-01-01</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
         <is>
           <t>milling_1</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>tool_milling</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>skill_milling</t>
         </is>
@@ -1085,7 +1242,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1096,23 +1253,26 @@
       <c r="E4" t="n">
         <v>6</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
         <is>
           <t>T-0001-01</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>assembly_1</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>tool_assembly</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>skill_assembly</t>
         </is>
@@ -1124,6 +1284,144 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>op_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>initial_status</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>initial_start_time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>initial_end_time</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>initial_remaining_processing_time</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>initial_assigned_machine_id</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>initial_assigned_tooling_ids</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>initial_assigned_personnel_ids</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>OP-0001-01-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Completed before the planning anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OP-0001-ASM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>processing</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>assembly_1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>TL-assembly-01</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>PS-assembly-01</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Currently running and occupying resources until hour 6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1162,7 +1460,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>车削</t>
+          <t>Turning</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1179,7 +1477,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>铣削</t>
+          <t>Milling</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1196,7 +1494,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>装配</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1210,7 +1508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1255,7 +1553,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>车床-1</t>
+          <t>Turning-1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1277,7 +1575,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>铣床-1</t>
+          <t>Milling-1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1299,7 +1597,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>装配工位-1</t>
+          <t>Assembly-1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1310,72 +1608,6 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>0/8/10</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>type_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>type_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>tool_turning</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>车削工装</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>tool_milling</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>铣削工装</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>tool_assembly</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>装配工装</t>
         </is>
       </c>
     </row>
@@ -1390,100 +1622,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>tooling_id</t>
+          <t>type_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>tooling_name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>type_id</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>shifts</t>
+          <t>type_name</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TL-turning-01</t>
+          <t>tool_turning</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>车削工装-1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>tool_turning</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0/8/10;0/20/8</t>
+          <t>Turning tooling</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TL-milling-01</t>
+          <t>tool_milling</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>铣削工装-1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>tool_milling</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0/8/10</t>
+          <t>Milling tooling</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TL-assembly-01</t>
+          <t>tool_assembly</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>装配工装-1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>tool_assembly</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>0/8/10</t>
+          <t>Assembly tooling</t>
         </is>
       </c>
     </row>
@@ -1502,25 +1692,25 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>personnel_id</t>
+          <t>tooling_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>personnel_name</t>
+          <t>tooling_name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>type_id</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1532,17 +1722,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PS-turning-01</t>
+          <t>TL-turning-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>车削操作工-1</t>
+          <t>Turning-tool-1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>skill_turning</t>
+          <t>tool_turning</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1554,17 +1744,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PS-milling-01</t>
+          <t>TL-milling-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>铣削操作工-1</t>
+          <t>Milling-tool-1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>skill_milling</t>
+          <t>tool_milling</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1576,17 +1766,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PS-assembly-01</t>
+          <t>TL-assembly-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>装配操作工-1</t>
+          <t>Assembly-tool-1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>skill_assembly</t>
+          <t>tool_assembly</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>